<commit_message>
feat: cancel online visual search/comparison, retain doodle studio (draw, upload photo, camera), and add comprehensive user manual
</commit_message>
<xml_diff>
--- a/test_screenshots/情緒觀察表統計報表_2026-10-31.xlsx
+++ b/test_screenshots/情緒觀察表統計報表_2026-10-31.xlsx
@@ -410,7 +410,7 @@
         <v>產生時間</v>
       </c>
       <c r="B2" t="str">
-        <v>10/31/2026, 8:50:26 AM</v>
+        <v>10/31/2026, 9:03:35 AM</v>
       </c>
     </row>
     <row r="3">
@@ -434,7 +434,7 @@
         <v>最強烈情緒</v>
       </c>
       <c r="B5" t="str">
-        <v>不解 94 / 6次</v>
+        <v>傻眼 94 / 6次</v>
       </c>
     </row>
     <row r="6">
@@ -450,7 +450,7 @@
         <v>最有效落地方式</v>
       </c>
       <c r="B7" t="str">
-        <v>按摩腸胃 71 / 1次</v>
+        <v>按摩腸胃 90 / 1次</v>
       </c>
     </row>
     <row r="8">
@@ -551,7 +551,7 @@
         <v>當下</v>
       </c>
       <c r="K2">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="L2" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -598,7 +598,7 @@
         <v>當下</v>
       </c>
       <c r="K3">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="L3" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -633,10 +633,10 @@
         <v>啊？</v>
       </c>
       <c r="G4" t="str">
-        <v>不喜(64)</v>
+        <v>不喜(77)</v>
       </c>
       <c r="H4">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="I4" t="str">
         <v>深呼吸</v>
@@ -645,7 +645,7 @@
         <v>當下</v>
       </c>
       <c r="K4">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="L4" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -680,10 +680,10 @@
         <v>啊？</v>
       </c>
       <c r="G5" t="str">
-        <v>傻眼(65)</v>
+        <v>傻眼(70)</v>
       </c>
       <c r="H5">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="I5" t="str">
         <v>深呼吸</v>
@@ -692,7 +692,7 @@
         <v>當下</v>
       </c>
       <c r="K5">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="L5" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -727,10 +727,10 @@
         <v>啊？</v>
       </c>
       <c r="G6" t="str">
-        <v>不解(88)</v>
+        <v>不解(82)</v>
       </c>
       <c r="H6">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="I6" t="str">
         <v>深呼吸</v>
@@ -774,10 +774,10 @@
         <v>啊？</v>
       </c>
       <c r="G7" t="str">
-        <v>不喜(62)</v>
+        <v>不喜(75)</v>
       </c>
       <c r="H7">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="I7" t="str">
         <v>深呼吸</v>
@@ -786,7 +786,7 @@
         <v>事後</v>
       </c>
       <c r="K7">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L7" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -821,10 +821,10 @@
         <v>啊？</v>
       </c>
       <c r="G8" t="str">
-        <v>傻眼(81)</v>
+        <v>傻眼(84)</v>
       </c>
       <c r="H8">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="I8" t="str">
         <v>深呼吸</v>
@@ -833,7 +833,7 @@
         <v>事後</v>
       </c>
       <c r="K8">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="L8" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -868,10 +868,10 @@
         <v>啊？</v>
       </c>
       <c r="G9" t="str">
-        <v>不解(94)</v>
+        <v>不解(92)</v>
       </c>
       <c r="H9">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I9" t="str">
         <v>深呼吸</v>
@@ -880,7 +880,7 @@
         <v>事後</v>
       </c>
       <c r="K9">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="L9" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -915,10 +915,10 @@
         <v>啊？</v>
       </c>
       <c r="G10" t="str">
-        <v>不喜(77)</v>
+        <v>不喜(83)</v>
       </c>
       <c r="H10">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="I10" t="str">
         <v>深呼吸</v>
@@ -927,7 +927,7 @@
         <v>事後</v>
       </c>
       <c r="K10">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="L10" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -962,10 +962,10 @@
         <v>啊？</v>
       </c>
       <c r="G11" t="str">
-        <v>傻眼(84)</v>
+        <v>傻眼(94)</v>
       </c>
       <c r="H11">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="I11" t="str">
         <v>深呼吸</v>
@@ -974,7 +974,7 @@
         <v>事後</v>
       </c>
       <c r="K11">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="L11" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1009,10 +1009,10 @@
         <v>啊？</v>
       </c>
       <c r="G12" t="str">
-        <v>不解(72)</v>
+        <v>不解(80)</v>
       </c>
       <c r="H12">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I12" t="str">
         <v>深呼吸</v>
@@ -1021,7 +1021,7 @@
         <v>事後</v>
       </c>
       <c r="K12">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="L12" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1056,10 +1056,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G13" t="str">
-        <v>不喜(62)</v>
+        <v>不喜(83)</v>
       </c>
       <c r="H13">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="I13" t="str">
         <v>深呼吸</v>
@@ -1068,7 +1068,7 @@
         <v>事後</v>
       </c>
       <c r="K13">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="L13" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1103,10 +1103,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G14" t="str">
-        <v>傻眼(72)</v>
+        <v>傻眼(67)</v>
       </c>
       <c r="H14">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I14" t="str">
         <v>深呼吸</v>
@@ -1115,7 +1115,7 @@
         <v>事後</v>
       </c>
       <c r="K14">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="L14" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1150,10 +1150,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G15" t="str">
-        <v>不解(60)</v>
+        <v>不解(64)</v>
       </c>
       <c r="H15">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I15" t="str">
         <v>深呼吸</v>
@@ -1162,7 +1162,7 @@
         <v>事後</v>
       </c>
       <c r="K15">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="L15" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1197,10 +1197,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G16" t="str">
-        <v>不喜(61)</v>
+        <v>不喜(62)</v>
       </c>
       <c r="H16">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I16" t="str">
         <v>深呼吸</v>
@@ -1209,7 +1209,7 @@
         <v>事後</v>
       </c>
       <c r="K16">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="L16" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1244,10 +1244,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G17" t="str">
-        <v>傻眼(91)</v>
+        <v>傻眼(64)</v>
       </c>
       <c r="H17">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="I17" t="str">
         <v>敲胸</v>
@@ -1256,7 +1256,7 @@
         <v>未落地</v>
       </c>
       <c r="K17">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="L17" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1291,10 +1291,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G18" t="str">
-        <v>不解(91)</v>
+        <v>不解(70)</v>
       </c>
       <c r="H18">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="I18" t="str">
         <v>敲胸</v>
@@ -1303,7 +1303,7 @@
         <v>未落地</v>
       </c>
       <c r="K18">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="L18" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1338,10 +1338,10 @@
         <v>糟糕</v>
       </c>
       <c r="G19" t="str">
-        <v>不喜(84)</v>
+        <v>不喜(61)</v>
       </c>
       <c r="H19">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="I19" t="str">
         <v>敲胸</v>
@@ -1350,7 +1350,7 @@
         <v>未落地</v>
       </c>
       <c r="K19">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="L19" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1385,10 +1385,10 @@
         <v>糟糕</v>
       </c>
       <c r="G20" t="str">
-        <v>傻眼(63)</v>
+        <v>傻眼(68)</v>
       </c>
       <c r="H20">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I20" t="str">
         <v>敲胸</v>
@@ -1397,7 +1397,7 @@
         <v>未落地</v>
       </c>
       <c r="K20">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="L20" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1432,10 +1432,10 @@
         <v>糟糕</v>
       </c>
       <c r="G21" t="str">
-        <v>不解(75)</v>
+        <v>不解(94)</v>
       </c>
       <c r="H21">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="I21" t="str">
         <v>按摩腸胃、腳踩大地</v>
@@ -1479,10 +1479,10 @@
         <v>糟糕</v>
       </c>
       <c r="G22" t="str">
-        <v>不喜(62)</v>
+        <v>不喜(87)</v>
       </c>
       <c r="H22">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="I22" t="str">
         <v>腳踩大地</v>
@@ -1491,7 +1491,7 @@
         <v>未落地</v>
       </c>
       <c r="K22">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="L22" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>

</xml_diff>

<commit_message>
feat: add multi-channel share for doodle canvas (native share, copy image to clipboard, Discord webhook push, and PNG download)
</commit_message>
<xml_diff>
--- a/test_screenshots/情緒觀察表統計報表_2026-10-31.xlsx
+++ b/test_screenshots/情緒觀察表統計報表_2026-10-31.xlsx
@@ -410,7 +410,7 @@
         <v>產生時間</v>
       </c>
       <c r="B2" t="str">
-        <v>10/31/2026, 9:03:35 AM</v>
+        <v>10/31/2026, 9:11:56 AM</v>
       </c>
     </row>
     <row r="3">
@@ -434,7 +434,7 @@
         <v>最強烈情緒</v>
       </c>
       <c r="B5" t="str">
-        <v>傻眼 94 / 6次</v>
+        <v>不喜 91 / 7次</v>
       </c>
     </row>
     <row r="6">
@@ -450,7 +450,7 @@
         <v>最有效落地方式</v>
       </c>
       <c r="B7" t="str">
-        <v>按摩腸胃 90 / 1次</v>
+        <v>按摩腸胃 65 / 1次</v>
       </c>
     </row>
     <row r="8">
@@ -551,7 +551,7 @@
         <v>當下</v>
       </c>
       <c r="K2">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="L2" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -598,7 +598,7 @@
         <v>當下</v>
       </c>
       <c r="K3">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="L3" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -633,10 +633,10 @@
         <v>啊？</v>
       </c>
       <c r="G4" t="str">
-        <v>不喜(77)</v>
+        <v>不喜(65)</v>
       </c>
       <c r="H4">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="I4" t="str">
         <v>深呼吸</v>
@@ -645,7 +645,7 @@
         <v>當下</v>
       </c>
       <c r="K4">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="L4" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -680,10 +680,10 @@
         <v>啊？</v>
       </c>
       <c r="G5" t="str">
-        <v>傻眼(70)</v>
+        <v>傻眼(87)</v>
       </c>
       <c r="H5">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="I5" t="str">
         <v>深呼吸</v>
@@ -692,7 +692,7 @@
         <v>當下</v>
       </c>
       <c r="K5">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="L5" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -727,10 +727,10 @@
         <v>啊？</v>
       </c>
       <c r="G6" t="str">
-        <v>不解(82)</v>
+        <v>不解(73)</v>
       </c>
       <c r="H6">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="I6" t="str">
         <v>深呼吸</v>
@@ -739,7 +739,7 @@
         <v>當下</v>
       </c>
       <c r="K6">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="L6" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -774,10 +774,10 @@
         <v>啊？</v>
       </c>
       <c r="G7" t="str">
-        <v>不喜(75)</v>
+        <v>不喜(88)</v>
       </c>
       <c r="H7">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="I7" t="str">
         <v>深呼吸</v>
@@ -821,10 +821,10 @@
         <v>啊？</v>
       </c>
       <c r="G8" t="str">
-        <v>傻眼(84)</v>
+        <v>傻眼(72)</v>
       </c>
       <c r="H8">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="I8" t="str">
         <v>深呼吸</v>
@@ -833,7 +833,7 @@
         <v>事後</v>
       </c>
       <c r="K8">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="L8" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -868,10 +868,10 @@
         <v>啊？</v>
       </c>
       <c r="G9" t="str">
-        <v>不解(92)</v>
+        <v>不解(84)</v>
       </c>
       <c r="H9">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="I9" t="str">
         <v>深呼吸</v>
@@ -880,7 +880,7 @@
         <v>事後</v>
       </c>
       <c r="K9">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="L9" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -915,10 +915,10 @@
         <v>啊？</v>
       </c>
       <c r="G10" t="str">
-        <v>不喜(83)</v>
+        <v>不喜(70)</v>
       </c>
       <c r="H10">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I10" t="str">
         <v>深呼吸</v>
@@ -927,7 +927,7 @@
         <v>事後</v>
       </c>
       <c r="K10">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L10" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -962,10 +962,10 @@
         <v>啊？</v>
       </c>
       <c r="G11" t="str">
-        <v>傻眼(94)</v>
+        <v>傻眼(64)</v>
       </c>
       <c r="H11">
-        <v>94</v>
+        <v>64</v>
       </c>
       <c r="I11" t="str">
         <v>深呼吸</v>
@@ -974,7 +974,7 @@
         <v>事後</v>
       </c>
       <c r="K11">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="L11" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1009,10 +1009,10 @@
         <v>啊？</v>
       </c>
       <c r="G12" t="str">
-        <v>不解(80)</v>
+        <v>不解(82)</v>
       </c>
       <c r="H12">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I12" t="str">
         <v>深呼吸</v>
@@ -1021,7 +1021,7 @@
         <v>事後</v>
       </c>
       <c r="K12">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="L12" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1056,10 +1056,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G13" t="str">
-        <v>不喜(83)</v>
+        <v>不喜(80)</v>
       </c>
       <c r="H13">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I13" t="str">
         <v>深呼吸</v>
@@ -1068,7 +1068,7 @@
         <v>事後</v>
       </c>
       <c r="K13">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="L13" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1103,10 +1103,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G14" t="str">
-        <v>傻眼(67)</v>
+        <v>傻眼(83)</v>
       </c>
       <c r="H14">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="I14" t="str">
         <v>深呼吸</v>
@@ -1115,7 +1115,7 @@
         <v>事後</v>
       </c>
       <c r="K14">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L14" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1150,10 +1150,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G15" t="str">
-        <v>不解(64)</v>
+        <v>不解(74)</v>
       </c>
       <c r="H15">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="I15" t="str">
         <v>深呼吸</v>
@@ -1162,7 +1162,7 @@
         <v>事後</v>
       </c>
       <c r="K15">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L15" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1197,10 +1197,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G16" t="str">
-        <v>不喜(62)</v>
+        <v>不喜(79)</v>
       </c>
       <c r="H16">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I16" t="str">
         <v>深呼吸</v>
@@ -1209,7 +1209,7 @@
         <v>事後</v>
       </c>
       <c r="K16">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L16" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1244,10 +1244,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G17" t="str">
-        <v>傻眼(64)</v>
+        <v>傻眼(83)</v>
       </c>
       <c r="H17">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="I17" t="str">
         <v>敲胸</v>
@@ -1256,7 +1256,7 @@
         <v>未落地</v>
       </c>
       <c r="K17">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="L17" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1291,10 +1291,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G18" t="str">
-        <v>不解(70)</v>
+        <v>不解(64)</v>
       </c>
       <c r="H18">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I18" t="str">
         <v>敲胸</v>
@@ -1303,7 +1303,7 @@
         <v>未落地</v>
       </c>
       <c r="K18">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="L18" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1338,10 +1338,10 @@
         <v>糟糕</v>
       </c>
       <c r="G19" t="str">
-        <v>不喜(61)</v>
+        <v>不喜(66)</v>
       </c>
       <c r="H19">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="I19" t="str">
         <v>敲胸</v>
@@ -1350,7 +1350,7 @@
         <v>未落地</v>
       </c>
       <c r="K19">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L19" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1385,10 +1385,10 @@
         <v>糟糕</v>
       </c>
       <c r="G20" t="str">
-        <v>傻眼(68)</v>
+        <v>傻眼(75)</v>
       </c>
       <c r="H20">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="I20" t="str">
         <v>敲胸</v>
@@ -1397,7 +1397,7 @@
         <v>未落地</v>
       </c>
       <c r="K20">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="L20" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1432,10 +1432,10 @@
         <v>糟糕</v>
       </c>
       <c r="G21" t="str">
-        <v>不解(94)</v>
+        <v>不解(69)</v>
       </c>
       <c r="H21">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="I21" t="str">
         <v>按摩腸胃、腳踩大地</v>
@@ -1479,10 +1479,10 @@
         <v>糟糕</v>
       </c>
       <c r="G22" t="str">
-        <v>不喜(87)</v>
+        <v>不喜(91)</v>
       </c>
       <c r="H22">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="I22" t="str">
         <v>腳踩大地</v>
@@ -1491,7 +1491,7 @@
         <v>未落地</v>
       </c>
       <c r="K22">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="L22" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>

</xml_diff>

<commit_message>
feat: add Body Awareness Silhouette Map, 15 emotion/sensation sticker stamps, and seamless freehand drawing as sketched in IMG_20261031_091636897_MFNR
</commit_message>
<xml_diff>
--- a/test_screenshots/情緒觀察表統計報表_2026-10-31.xlsx
+++ b/test_screenshots/情緒觀察表統計報表_2026-10-31.xlsx
@@ -410,7 +410,7 @@
         <v>產生時間</v>
       </c>
       <c r="B2" t="str">
-        <v>10/31/2026, 9:11:56 AM</v>
+        <v>10/31/2026, 9:39:09 AM</v>
       </c>
     </row>
     <row r="3">
@@ -434,7 +434,7 @@
         <v>最強烈情緒</v>
       </c>
       <c r="B5" t="str">
-        <v>不喜 91 / 7次</v>
+        <v>不喜 92 / 7次</v>
       </c>
     </row>
     <row r="6">
@@ -450,7 +450,7 @@
         <v>最有效落地方式</v>
       </c>
       <c r="B7" t="str">
-        <v>按摩腸胃 65 / 1次</v>
+        <v>按摩腸胃 80 / 1次</v>
       </c>
     </row>
     <row r="8">
@@ -551,7 +551,7 @@
         <v>當下</v>
       </c>
       <c r="K2">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="L2" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -598,7 +598,7 @@
         <v>當下</v>
       </c>
       <c r="K3">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="L3" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -633,10 +633,10 @@
         <v>啊？</v>
       </c>
       <c r="G4" t="str">
-        <v>不喜(65)</v>
+        <v>不喜(78)</v>
       </c>
       <c r="H4">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="I4" t="str">
         <v>深呼吸</v>
@@ -645,7 +645,7 @@
         <v>當下</v>
       </c>
       <c r="K4">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="L4" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -680,10 +680,10 @@
         <v>啊？</v>
       </c>
       <c r="G5" t="str">
-        <v>傻眼(87)</v>
+        <v>傻眼(63)</v>
       </c>
       <c r="H5">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="I5" t="str">
         <v>深呼吸</v>
@@ -692,7 +692,7 @@
         <v>當下</v>
       </c>
       <c r="K5">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="L5" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -727,10 +727,10 @@
         <v>啊？</v>
       </c>
       <c r="G6" t="str">
-        <v>不解(73)</v>
+        <v>不解(67)</v>
       </c>
       <c r="H6">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="I6" t="str">
         <v>深呼吸</v>
@@ -739,7 +739,7 @@
         <v>當下</v>
       </c>
       <c r="K6">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L6" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -774,10 +774,10 @@
         <v>啊？</v>
       </c>
       <c r="G7" t="str">
-        <v>不喜(88)</v>
+        <v>不喜(81)</v>
       </c>
       <c r="H7">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I7" t="str">
         <v>深呼吸</v>
@@ -786,7 +786,7 @@
         <v>事後</v>
       </c>
       <c r="K7">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L7" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -821,10 +821,10 @@
         <v>啊？</v>
       </c>
       <c r="G8" t="str">
-        <v>傻眼(72)</v>
+        <v>傻眼(79)</v>
       </c>
       <c r="H8">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I8" t="str">
         <v>深呼吸</v>
@@ -833,7 +833,7 @@
         <v>事後</v>
       </c>
       <c r="K8">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="L8" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -868,10 +868,10 @@
         <v>啊？</v>
       </c>
       <c r="G9" t="str">
-        <v>不解(84)</v>
+        <v>不解(60)</v>
       </c>
       <c r="H9">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="I9" t="str">
         <v>深呼吸</v>
@@ -880,7 +880,7 @@
         <v>事後</v>
       </c>
       <c r="K9">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="L9" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -915,10 +915,10 @@
         <v>啊？</v>
       </c>
       <c r="G10" t="str">
-        <v>不喜(70)</v>
+        <v>不喜(75)</v>
       </c>
       <c r="H10">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I10" t="str">
         <v>深呼吸</v>
@@ -927,7 +927,7 @@
         <v>事後</v>
       </c>
       <c r="K10">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L10" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -962,10 +962,10 @@
         <v>啊？</v>
       </c>
       <c r="G11" t="str">
-        <v>傻眼(64)</v>
+        <v>傻眼(90)</v>
       </c>
       <c r="H11">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="I11" t="str">
         <v>深呼吸</v>
@@ -974,7 +974,7 @@
         <v>事後</v>
       </c>
       <c r="K11">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="L11" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1009,10 +1009,10 @@
         <v>啊？</v>
       </c>
       <c r="G12" t="str">
-        <v>不解(82)</v>
+        <v>不解(61)</v>
       </c>
       <c r="H12">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="I12" t="str">
         <v>深呼吸</v>
@@ -1021,7 +1021,7 @@
         <v>事後</v>
       </c>
       <c r="K12">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="L12" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1056,10 +1056,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G13" t="str">
-        <v>不喜(80)</v>
+        <v>不喜(83)</v>
       </c>
       <c r="H13">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I13" t="str">
         <v>深呼吸</v>
@@ -1068,7 +1068,7 @@
         <v>事後</v>
       </c>
       <c r="K13">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L13" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1103,10 +1103,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G14" t="str">
-        <v>傻眼(83)</v>
+        <v>傻眼(79)</v>
       </c>
       <c r="H14">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I14" t="str">
         <v>深呼吸</v>
@@ -1115,7 +1115,7 @@
         <v>事後</v>
       </c>
       <c r="K14">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L14" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1150,10 +1150,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G15" t="str">
-        <v>不解(74)</v>
+        <v>不解(78)</v>
       </c>
       <c r="H15">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="I15" t="str">
         <v>深呼吸</v>
@@ -1162,7 +1162,7 @@
         <v>事後</v>
       </c>
       <c r="K15">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="L15" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1197,10 +1197,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G16" t="str">
-        <v>不喜(79)</v>
+        <v>不喜(65)</v>
       </c>
       <c r="H16">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="I16" t="str">
         <v>深呼吸</v>
@@ -1209,7 +1209,7 @@
         <v>事後</v>
       </c>
       <c r="K16">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="L16" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1244,10 +1244,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G17" t="str">
-        <v>傻眼(83)</v>
+        <v>傻眼(85)</v>
       </c>
       <c r="H17">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I17" t="str">
         <v>敲胸</v>
@@ -1256,7 +1256,7 @@
         <v>未落地</v>
       </c>
       <c r="K17">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L17" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1291,10 +1291,10 @@
         <v>怎麼會這樣</v>
       </c>
       <c r="G18" t="str">
-        <v>不解(64)</v>
+        <v>不解(80)</v>
       </c>
       <c r="H18">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="I18" t="str">
         <v>敲胸</v>
@@ -1303,7 +1303,7 @@
         <v>未落地</v>
       </c>
       <c r="K18">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L18" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1338,10 +1338,10 @@
         <v>糟糕</v>
       </c>
       <c r="G19" t="str">
-        <v>不喜(66)</v>
+        <v>不喜(70)</v>
       </c>
       <c r="H19">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="I19" t="str">
         <v>敲胸</v>
@@ -1350,7 +1350,7 @@
         <v>未落地</v>
       </c>
       <c r="K19">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="L19" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>
@@ -1385,10 +1385,10 @@
         <v>糟糕</v>
       </c>
       <c r="G20" t="str">
-        <v>傻眼(75)</v>
+        <v>傻眼(84)</v>
       </c>
       <c r="H20">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="I20" t="str">
         <v>敲胸</v>
@@ -1432,10 +1432,10 @@
         <v>糟糕</v>
       </c>
       <c r="G21" t="str">
-        <v>不解(69)</v>
+        <v>不解(84)</v>
       </c>
       <c r="H21">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="I21" t="str">
         <v>按摩腸胃、腳踩大地</v>
@@ -1479,10 +1479,10 @@
         <v>糟糕</v>
       </c>
       <c r="G22" t="str">
-        <v>不喜(91)</v>
+        <v>不喜(92)</v>
       </c>
       <c r="H22">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I22" t="str">
         <v>腳踩大地</v>
@@ -1491,7 +1491,7 @@
         <v>未落地</v>
       </c>
       <c r="K22">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="L22" t="str">
         <v>以為對方故意找麻煩或事情徹底搞砸了</v>

</xml_diff>